<commit_message>
perf(ohscanner): report fixed-corpus incremental comparison
</commit_message>
<xml_diff>
--- a/research/deliveries/performance/full_efficiency_20261021/OHScanner_Efficiency_E0-E4_20261021.xlsx
+++ b/research/deliveries/performance/full_efficiency_20261021/OHScanner_Efficiency_E0-E4_20261021.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E0-E4对照" sheetId="1" r:id="Reab9613f82114b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前后指标" sheetId="2" r:id="Rd8431343a10348a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计与边界" sheetId="3" r:id="R4462e58ddde04bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P3 current" sheetId="4" r:id="R3c5525d5c7ee4e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 cache" sheetId="5" r:id="R5a78e478aa964640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 fixed corpus" sheetId="6" r:id="Rcaa5695f6dc44445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 M2 固定语料" sheetId="7" r:id="Ra9572c189e004a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E0-E4对照" sheetId="1" r:id="R276c10918906410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前后指标" sheetId="2" r:id="Rf8bc44fb29174ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计与边界" sheetId="3" r:id="R30bf853218d04bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P3 current" sheetId="4" r:id="Ra1f77657bd0e43bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 cache" sheetId="5" r:id="R5942353215e44072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 fixed corpus" sheetId="6" r:id="Rcf5f94a0dc2545f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 M2 固定语料" sheetId="7" r:id="R77bfe86b45fc459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2 fixed corpus" sheetId="8" r:id="R9949ed584c1d4009"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +25,7 @@
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -109,8 +110,14 @@
       <x:color rgb="FF243244"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="8"/>
+      <x:color rgb="FF243244"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="88">
+  <x:fills count="114">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -545,6 +552,136 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -589,7 +726,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="248">
+  <x:cellXfs count="354">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -1183,6 +1320,298 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="95" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="97" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="97" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="98" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="97" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="99" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="97" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="96" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="100" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="102" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="100" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="103" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="100" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="100" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="101" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="105" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="105" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="106" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="105" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="105" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="104" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="108" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="108" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="108" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="104" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="104" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="104" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="105" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="105" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="105" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="111" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="112" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="110" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="113" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="113" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="113" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="113" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="109" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="109" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="109" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="110" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="110" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="110" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1597,44 +2026,32 @@
         <x:v>三文件样本：仅扫变更文件漏掉 3/3 个未变文件候选；不作为完整扫描或性能结果</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="52" customHeight="1">
+    <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">E2</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">依赖规划 + 不安全时全量回退</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">unit validated; corpus not_run</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">unknown</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">unknown</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">unknown</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0 reused</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H6" s="154" t="str">
-        <x:v>first-parent SHA 已取得；bare fetch 无法连接 GitHub；C/C++ call 闭包与 base AST cache；跨语言或歧义时仍全量扫描</x:v>
+      <x:c r="B6" s="155" t="str">
+        <x:v>base→head；变更配置时保守全量回退，复用已声明的完整单文件 detector 结果</x:v>
+      </x:c>
+      <x:c r="C6" s="155" t="str">
+        <x:v>固定语料 E2 冷/热已完成；11/11 等价</x:v>
+      </x:c>
+      <x:c r="D6" s="253" t="n">
+        <x:v>66.61789999999999</x:v>
+      </x:c>
+      <x:c r="E6" s="253" t="n">
+        <x:v>30.949750000000005</x:v>
+      </x:c>
+      <x:c r="F6" s="253" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="G6" s="253" t="n">
+        <x:v>333552</x:v>
+      </x:c>
+      <x:c r="H6" s="155" t="str">
+        <x:v>同环境 E0=94.8s；E2 冷=164.6s，热=66.6s（热 vs E0 -29.7%）。热缓存未减少扫描覆盖；所有组件仍 completed_with_limitations。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2827,20 +3244,20 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="239" t="str">
+      <x:c r="A1" s="335" t="str">
         <x:v>P2 单文件检测结果缓存：固定 11 组件冷/热对照</x:v>
       </x:c>
-      <x:c r="B1" s="239"/>
-      <x:c r="C1" s="239"/>
-      <x:c r="D1" s="239"/>
-      <x:c r="E1" s="239"/>
-      <x:c r="F1" s="239"/>
-      <x:c r="G1" s="239"/>
-      <x:c r="H1" s="239"/>
-      <x:c r="I1" s="239"/>
-      <x:c r="J1" s="239"/>
-      <x:c r="K1" s="239"/>
-      <x:c r="L1" s="239"/>
+      <x:c r="B1" s="335"/>
+      <x:c r="C1" s="335"/>
+      <x:c r="D1" s="335"/>
+      <x:c r="E1" s="335"/>
+      <x:c r="F1" s="335"/>
+      <x:c r="G1" s="335"/>
+      <x:c r="H1" s="335"/>
+      <x:c r="I1" s="335"/>
+      <x:c r="J1" s="335"/>
+      <x:c r="K1" s="335"/>
+      <x:c r="L1" s="335"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="16" t="str">
@@ -2859,40 +3276,40 @@
       <x:c r="L2" s="16"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="240" t="str">
+      <x:c r="A4" s="336" t="str">
         <x:v>实验</x:v>
       </x:c>
-      <x:c r="B4" s="240" t="str">
+      <x:c r="B4" s="336" t="str">
         <x:v>模式</x:v>
       </x:c>
-      <x:c r="C4" s="240" t="str">
+      <x:c r="C4" s="336" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="D4" s="240" t="str">
+      <x:c r="D4" s="336" t="str">
         <x:v>总墙钟秒</x:v>
       </x:c>
-      <x:c r="E4" s="240" t="str">
+      <x:c r="E4" s="336" t="str">
         <x:v>进程 CPU 秒</x:v>
       </x:c>
-      <x:c r="F4" s="240" t="str">
+      <x:c r="F4" s="336" t="str">
         <x:v>AST 墙钟秒</x:v>
       </x:c>
-      <x:c r="G4" s="240" t="str">
+      <x:c r="G4" s="336" t="str">
         <x:v>AST CPU 秒</x:v>
       </x:c>
-      <x:c r="H4" s="240" t="str">
+      <x:c r="H4" s="336" t="str">
         <x:v>解析文件数</x:v>
       </x:c>
-      <x:c r="I4" s="240" t="str">
+      <x:c r="I4" s="336" t="str">
         <x:v>结果缓存 hit / miss</x:v>
       </x:c>
-      <x:c r="J4" s="240" t="str">
+      <x:c r="J4" s="336" t="str">
         <x:v>Detector 阶段墙钟秒</x:v>
       </x:c>
-      <x:c r="K4" s="240" t="str">
+      <x:c r="K4" s="336" t="str">
         <x:v>峰值 RSS KB</x:v>
       </x:c>
-      <x:c r="L4" s="240" t="str">
+      <x:c r="L4" s="336" t="str">
         <x:v>结果等价</x:v>
       </x:c>
     </x:row>
@@ -3011,13 +3428,13 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="241" t="str">
+      <x:c r="A9" s="337" t="str">
         <x:v>核对</x:v>
       </x:c>
-      <x:c r="B9" s="241" t="str">
+      <x:c r="B9" s="337" t="str">
         <x:v>实测</x:v>
       </x:c>
-      <x:c r="C9" s="241" t="str">
+      <x:c r="C9" s="337" t="str">
         <x:v>解释</x:v>
       </x:c>
     </x:row>
@@ -3121,36 +3538,36 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
-      <x:c r="A20" s="242" t="str">
+      <x:c r="A20" s="338" t="str">
         <x:v>结论：输出等价通过，但该 detector-result cache 反而显著变慢，AST 解析 CPU 不变；仅保持 opt-in 研究状态，不作为性能收益交付。P0/P1 AST summary cache 是减少重复 AST 解析的实现，数据另见 P3 current 页。示例 detector 不是 ABCD 全量漏洞扫描。</x:v>
       </x:c>
-      <x:c r="B20" s="242"/>
-      <x:c r="C20" s="242"/>
-      <x:c r="D20" s="242"/>
-      <x:c r="E20" s="242"/>
-      <x:c r="F20" s="242"/>
-      <x:c r="G20" s="242"/>
-      <x:c r="H20" s="242"/>
-      <x:c r="I20" s="242"/>
-      <x:c r="J20" s="242"/>
-      <x:c r="K20" s="242"/>
-      <x:c r="L20" s="242"/>
+      <x:c r="B20" s="338"/>
+      <x:c r="C20" s="338"/>
+      <x:c r="D20" s="338"/>
+      <x:c r="E20" s="338"/>
+      <x:c r="F20" s="338"/>
+      <x:c r="G20" s="338"/>
+      <x:c r="H20" s="338"/>
+      <x:c r="I20" s="338"/>
+      <x:c r="J20" s="338"/>
+      <x:c r="K20" s="338"/>
+      <x:c r="L20" s="338"/>
     </x:row>
     <x:row r="22" ht="27" customHeight="1">
-      <x:c r="A22" s="243" t="str">
+      <x:c r="A22" s="339" t="str">
         <x:v>Workbench 增量基线接口与边界</x:v>
       </x:c>
-      <x:c r="B22" s="243"/>
-      <x:c r="C22" s="243"/>
-      <x:c r="D22" s="243"/>
-      <x:c r="E22" s="243"/>
-      <x:c r="F22" s="243"/>
-      <x:c r="G22" s="243"/>
-      <x:c r="H22" s="243"/>
-      <x:c r="I22" s="243"/>
-      <x:c r="J22" s="243"/>
-      <x:c r="K22" s="243"/>
-      <x:c r="L22" s="243"/>
+      <x:c r="B22" s="339"/>
+      <x:c r="C22" s="339"/>
+      <x:c r="D22" s="339"/>
+      <x:c r="E22" s="339"/>
+      <x:c r="F22" s="339"/>
+      <x:c r="G22" s="339"/>
+      <x:c r="H22" s="339"/>
+      <x:c r="I22" s="339"/>
+      <x:c r="J22" s="339"/>
+      <x:c r="K22" s="339"/>
+      <x:c r="L22" s="339"/>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
       <x:c r="A23" s="39" t="str">
@@ -3243,20 +3660,20 @@
       <x:c r="L27" s="31"/>
     </x:row>
     <x:row r="29" ht="27" customHeight="1">
-      <x:c r="A29" s="243" t="str">
+      <x:c r="A29" s="339" t="str">
         <x:v>P4 中途 detector 分片检查点与恢复验证</x:v>
       </x:c>
-      <x:c r="B29" s="243"/>
-      <x:c r="C29" s="243"/>
-      <x:c r="D29" s="243"/>
-      <x:c r="E29" s="243"/>
-      <x:c r="F29" s="243"/>
-      <x:c r="G29" s="243"/>
-      <x:c r="H29" s="243"/>
-      <x:c r="I29" s="243"/>
-      <x:c r="J29" s="243"/>
-      <x:c r="K29" s="243"/>
-      <x:c r="L29" s="243"/>
+      <x:c r="B29" s="339"/>
+      <x:c r="C29" s="339"/>
+      <x:c r="D29" s="339"/>
+      <x:c r="E29" s="339"/>
+      <x:c r="F29" s="339"/>
+      <x:c r="G29" s="339"/>
+      <x:c r="H29" s="339"/>
+      <x:c r="I29" s="339"/>
+      <x:c r="J29" s="339"/>
+      <x:c r="K29" s="339"/>
+      <x:c r="L29" s="339"/>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="39" t="str">
@@ -3431,77 +3848,77 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="244" t="str">
+      <x:c r="A1" s="340" t="str">
         <x:v>P2：M2 两个逐文件 detector 的固定 11 组件缓存对照</x:v>
       </x:c>
-      <x:c r="B1" s="244"/>
-      <x:c r="C1" s="244"/>
-      <x:c r="D1" s="244"/>
-      <x:c r="E1" s="244"/>
-      <x:c r="F1" s="244"/>
-      <x:c r="G1" s="244"/>
-      <x:c r="H1" s="244"/>
-      <x:c r="I1" s="244"/>
-      <x:c r="J1" s="244"/>
-      <x:c r="K1" s="244"/>
-      <x:c r="L1" s="244"/>
-      <x:c r="M1" s="244"/>
+      <x:c r="B1" s="340"/>
+      <x:c r="C1" s="340"/>
+      <x:c r="D1" s="340"/>
+      <x:c r="E1" s="340"/>
+      <x:c r="F1" s="340"/>
+      <x:c r="G1" s="340"/>
+      <x:c r="H1" s="340"/>
+      <x:c r="I1" s="340"/>
+      <x:c r="J1" s="340"/>
+      <x:c r="K1" s="340"/>
+      <x:c r="L1" s="340"/>
+      <x:c r="M1" s="340"/>
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
-      <x:c r="A2" s="245" t="str">
+      <x:c r="A2" s="341" t="str">
         <x:v>固定 9,508 个源码文件；候选执行成本实验，不是漏洞准确率或 ABCD 全量扫描。E3 缓存位于 WSL2 ext4；所有组候选/位置/解析/覆盖/状态签名需与 E0 一致。所有 11 个 head SHA 匹配 manifest，但 parent commit 对象 0/11 可用，完整 E2 base→head 语料对照未运行。</x:v>
       </x:c>
-      <x:c r="B2" s="245"/>
-      <x:c r="C2" s="245"/>
-      <x:c r="D2" s="245"/>
-      <x:c r="E2" s="245"/>
-      <x:c r="F2" s="245"/>
-      <x:c r="G2" s="245"/>
-      <x:c r="H2" s="245"/>
-      <x:c r="I2" s="245"/>
-      <x:c r="J2" s="245"/>
-      <x:c r="K2" s="245"/>
-      <x:c r="L2" s="245"/>
-      <x:c r="M2" s="245"/>
+      <x:c r="B2" s="341"/>
+      <x:c r="C2" s="341"/>
+      <x:c r="D2" s="341"/>
+      <x:c r="E2" s="341"/>
+      <x:c r="F2" s="341"/>
+      <x:c r="G2" s="341"/>
+      <x:c r="H2" s="341"/>
+      <x:c r="I2" s="341"/>
+      <x:c r="J2" s="341"/>
+      <x:c r="K2" s="341"/>
+      <x:c r="L2" s="341"/>
+      <x:c r="M2" s="341"/>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="240" t="str">
+      <x:c r="A4" s="336" t="str">
         <x:v>实验组</x:v>
       </x:c>
-      <x:c r="B4" s="240" t="str">
+      <x:c r="B4" s="336" t="str">
         <x:v>总墙钟秒</x:v>
       </x:c>
-      <x:c r="C4" s="240" t="str">
+      <x:c r="C4" s="336" t="str">
         <x:v>进程 CPU 秒</x:v>
       </x:c>
-      <x:c r="D4" s="240" t="str">
+      <x:c r="D4" s="336" t="str">
         <x:v>AST CPU 秒</x:v>
       </x:c>
-      <x:c r="E4" s="240" t="str">
+      <x:c r="E4" s="336" t="str">
         <x:v>Detector 阶段秒</x:v>
       </x:c>
-      <x:c r="F4" s="240" t="str">
+      <x:c r="F4" s="336" t="str">
         <x:v>Parser 调用文件</x:v>
       </x:c>
-      <x:c r="G4" s="240" t="str">
+      <x:c r="G4" s="336" t="str">
         <x:v>AST cache hit</x:v>
       </x:c>
-      <x:c r="H4" s="240" t="str">
+      <x:c r="H4" s="336" t="str">
         <x:v>结果 cache hit</x:v>
       </x:c>
-      <x:c r="I4" s="240" t="str">
+      <x:c r="I4" s="336" t="str">
         <x:v>结果 cache miss</x:v>
       </x:c>
-      <x:c r="J4" s="240" t="str">
+      <x:c r="J4" s="336" t="str">
         <x:v>候选数</x:v>
       </x:c>
-      <x:c r="K4" s="240" t="str">
+      <x:c r="K4" s="336" t="str">
         <x:v>峰值 RSS KB</x:v>
       </x:c>
-      <x:c r="L4" s="240" t="str">
+      <x:c r="L4" s="336" t="str">
         <x:v>整体状态</x:v>
       </x:c>
-      <x:c r="M4" s="240" t="str">
+      <x:c r="M4" s="336" t="str">
         <x:v>结果等价</x:v>
       </x:c>
     </x:row>
@@ -3670,16 +4087,16 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="246" t="str">
+      <x:c r="A10" s="342" t="str">
         <x:v>关键对照</x:v>
       </x:c>
-      <x:c r="B10" s="246" t="str">
+      <x:c r="B10" s="342" t="str">
         <x:v>实测变化</x:v>
       </x:c>
-      <x:c r="C10" s="246" t="str">
+      <x:c r="C10" s="342" t="str">
         <x:v>解释</x:v>
       </x:c>
-      <x:c r="D10" s="246" t="str">
+      <x:c r="D10" s="342" t="str">
         <x:v>边界</x:v>
       </x:c>
     </x:row>
@@ -3768,60 +4185,60 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
-      <x:c r="A17" s="247" t="str">
+      <x:c r="A17" s="343" t="str">
         <x:v>逐组件原始对照：每行一个组件/实验组；result signature 绑定诊断、源码定位、解析、检测器覆盖和整体状态。</x:v>
       </x:c>
-      <x:c r="B17" s="247"/>
-      <x:c r="C17" s="247"/>
-      <x:c r="D17" s="247"/>
-      <x:c r="E17" s="247"/>
-      <x:c r="F17" s="247"/>
-      <x:c r="G17" s="247"/>
-      <x:c r="H17" s="247"/>
-      <x:c r="I17" s="247"/>
-      <x:c r="J17" s="247"/>
-      <x:c r="K17" s="247"/>
-      <x:c r="L17" s="247"/>
-      <x:c r="M17" s="247"/>
+      <x:c r="B17" s="343"/>
+      <x:c r="C17" s="343"/>
+      <x:c r="D17" s="343"/>
+      <x:c r="E17" s="343"/>
+      <x:c r="F17" s="343"/>
+      <x:c r="G17" s="343"/>
+      <x:c r="H17" s="343"/>
+      <x:c r="I17" s="343"/>
+      <x:c r="J17" s="343"/>
+      <x:c r="K17" s="343"/>
+      <x:c r="L17" s="343"/>
+      <x:c r="M17" s="343"/>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
-      <x:c r="A18" s="240" t="str">
+      <x:c r="A18" s="336" t="str">
         <x:v>组件</x:v>
       </x:c>
-      <x:c r="B18" s="240" t="str">
+      <x:c r="B18" s="336" t="str">
         <x:v>实验组</x:v>
       </x:c>
-      <x:c r="C18" s="240" t="str">
+      <x:c r="C18" s="336" t="str">
         <x:v>固定 commit</x:v>
       </x:c>
-      <x:c r="D18" s="240" t="str">
+      <x:c r="D18" s="336" t="str">
         <x:v>墙钟秒</x:v>
       </x:c>
-      <x:c r="E18" s="240" t="str">
+      <x:c r="E18" s="336" t="str">
         <x:v>进程 CPU 秒</x:v>
       </x:c>
-      <x:c r="F18" s="240" t="str">
+      <x:c r="F18" s="336" t="str">
         <x:v>AST CPU 秒</x:v>
       </x:c>
-      <x:c r="G18" s="240" t="str">
+      <x:c r="G18" s="336" t="str">
         <x:v>Detector 阶段秒</x:v>
       </x:c>
-      <x:c r="H18" s="240" t="str">
+      <x:c r="H18" s="336" t="str">
         <x:v>Parser 调用</x:v>
       </x:c>
-      <x:c r="I18" s="240" t="str">
+      <x:c r="I18" s="336" t="str">
         <x:v>AST hit</x:v>
       </x:c>
-      <x:c r="J18" s="240" t="str">
+      <x:c r="J18" s="336" t="str">
         <x:v>结果 hit/miss</x:v>
       </x:c>
-      <x:c r="K18" s="240" t="str">
+      <x:c r="K18" s="336" t="str">
         <x:v>候选数</x:v>
       </x:c>
-      <x:c r="L18" s="240" t="str">
+      <x:c r="L18" s="336" t="str">
         <x:v>整体状态</x:v>
       </x:c>
-      <x:c r="M18" s="240" t="str">
+      <x:c r="M18" s="336" t="str">
         <x:v>与 E0 等价</x:v>
       </x:c>
     </x:row>
@@ -5637,4 +6054,1982 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF17365D"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="42" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="340" t="str">
+        <x:v>E2：固定 11 组件 base→head 与热缓存对照</x:v>
+      </x:c>
+      <x:c r="B1" s="340"/>
+      <x:c r="C1" s="340"/>
+      <x:c r="D1" s="340"/>
+      <x:c r="E1" s="340"/>
+      <x:c r="F1" s="340"/>
+      <x:c r="G1" s="340"/>
+      <x:c r="H1" s="340"/>
+      <x:c r="I1" s="340"/>
+      <x:c r="J1" s="340"/>
+      <x:c r="K1" s="340"/>
+      <x:c r="L1" s="340"/>
+      <x:c r="M1" s="340"/>
+      <x:c r="N1" s="340"/>
+    </x:row>
+    <x:row r="2" ht="48" customHeight="1">
+      <x:c r="A2" s="341" t="str">
+        <x:v>同环境 WSL2 / Python 3.14，11 个固定 head/base、9,508 个源码文件、两个 M2 detector。E2 冷/热缓存位于 WSL 原生 /tmp ext4；命中复用已声明可缓存的完整单文件 detector 结果，依赖或构建配置不完整时仍全量检查 head。不是 ABCD 全量扫描或准确率实验。</x:v>
+      </x:c>
+      <x:c r="B2" s="341"/>
+      <x:c r="C2" s="341"/>
+      <x:c r="D2" s="341"/>
+      <x:c r="E2" s="341"/>
+      <x:c r="F2" s="341"/>
+      <x:c r="G2" s="341"/>
+      <x:c r="H2" s="341"/>
+      <x:c r="I2" s="341"/>
+      <x:c r="J2" s="341"/>
+      <x:c r="K2" s="341"/>
+      <x:c r="L2" s="341"/>
+      <x:c r="M2" s="341"/>
+      <x:c r="N2" s="341"/>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="336" t="str">
+        <x:v>实验组</x:v>
+      </x:c>
+      <x:c r="B4" s="336" t="str">
+        <x:v>墙钟秒</x:v>
+      </x:c>
+      <x:c r="C4" s="336" t="str">
+        <x:v>进程 CPU 秒</x:v>
+      </x:c>
+      <x:c r="D4" s="336" t="str">
+        <x:v>AST CPU 秒</x:v>
+      </x:c>
+      <x:c r="E4" s="336" t="str">
+        <x:v>Detector 阶段秒</x:v>
+      </x:c>
+      <x:c r="F4" s="336" t="str">
+        <x:v>扫描文件清单</x:v>
+      </x:c>
+      <x:c r="G4" s="336" t="str">
+        <x:v>Parser 调用</x:v>
+      </x:c>
+      <x:c r="H4" s="336" t="str">
+        <x:v>AST hit</x:v>
+      </x:c>
+      <x:c r="I4" s="336" t="str">
+        <x:v>结果 hit</x:v>
+      </x:c>
+      <x:c r="J4" s="336" t="str">
+        <x:v>结果 miss</x:v>
+      </x:c>
+      <x:c r="K4" s="336" t="str">
+        <x:v>候选诊断</x:v>
+      </x:c>
+      <x:c r="L4" s="336" t="str">
+        <x:v>最大组件 RSS KB</x:v>
+      </x:c>
+      <x:c r="M4" s="336" t="str">
+        <x:v>等价/覆盖</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="29" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="B5" s="32" t="n">
+        <x:v>94.8001</x:v>
+      </x:c>
+      <x:c r="C5" s="32" t="n">
+        <x:v>81.636422</x:v>
+      </x:c>
+      <x:c r="D5" s="32" t="n">
+        <x:v>33.88353307399999</x:v>
+      </x:c>
+      <x:c r="E5" s="32" t="n">
+        <x:v>40.82793907900009</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="n">
+        <x:v>9508</x:v>
+      </x:c>
+      <x:c r="G5" s="35" t="n">
+        <x:v>9508</x:v>
+      </x:c>
+      <x:c r="H5" s="35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="35" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="L5" s="35" t="n">
+        <x:v>206476</x:v>
+      </x:c>
+      <x:c r="M5" s="29" t="str">
+        <x:v>11/11 completed；11/11 completed_with_limitations；11/11 签名一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="30" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="B6" s="33" t="n">
+        <x:v>164.627</x:v>
+      </x:c>
+      <x:c r="C6" s="33" t="n">
+        <x:v>121.324781</x:v>
+      </x:c>
+      <x:c r="D6" s="33" t="n">
+        <x:v>36.62076058000004</x:v>
+      </x:c>
+      <x:c r="E6" s="33" t="n">
+        <x:v>65.11852187200003</x:v>
+      </x:c>
+      <x:c r="F6" s="36" t="n">
+        <x:v>9508</x:v>
+      </x:c>
+      <x:c r="G6" s="36" t="n">
+        <x:v>9478</x:v>
+      </x:c>
+      <x:c r="H6" s="36" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I6" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="36" t="n">
+        <x:v>13144</x:v>
+      </x:c>
+      <x:c r="K6" s="36" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="L6" s="36" t="n">
+        <x:v>336376</x:v>
+      </x:c>
+      <x:c r="M6" s="30" t="str">
+        <x:v>11/11 completed；11/11 completed_with_limitations；11/11 签名一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="31" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="B7" s="34" t="n">
+        <x:v>66.61789999999999</x:v>
+      </x:c>
+      <x:c r="C7" s="34" t="n">
+        <x:v>30.949750000000005</x:v>
+      </x:c>
+      <x:c r="D7" s="34" t="n">
+        <x:v>1.3919759380000005</x:v>
+      </x:c>
+      <x:c r="E7" s="34" t="n">
+        <x:v>19.75486655999999</x:v>
+      </x:c>
+      <x:c r="F7" s="37" t="n">
+        <x:v>9508</x:v>
+      </x:c>
+      <x:c r="G7" s="37" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="H7" s="37" t="n">
+        <x:v>9307</x:v>
+      </x:c>
+      <x:c r="I7" s="37" t="n">
+        <x:v>13037</x:v>
+      </x:c>
+      <x:c r="J7" s="37" t="n">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="K7" s="37" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="L7" s="37" t="n">
+        <x:v>333552</x:v>
+      </x:c>
+      <x:c r="M7" s="31" t="str">
+        <x:v>11/11 completed；11/11 completed_with_limitations；11/11 签名一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="342" t="str">
+        <x:v>对照指标</x:v>
+      </x:c>
+      <x:c r="B9" s="342" t="str">
+        <x:v>E2 热 vs E0</x:v>
+      </x:c>
+      <x:c r="C9" s="342" t="str">
+        <x:v>E2 冷 vs E0</x:v>
+      </x:c>
+      <x:c r="D9" s="342" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="344" t="str">
+        <x:v>总墙钟</x:v>
+      </x:c>
+      <x:c r="B10" s="344" t="str">
+        <x:v>-29.7%</x:v>
+      </x:c>
+      <x:c r="C10" s="344" t="str">
+        <x:v>73.7%</x:v>
+      </x:c>
+      <x:c r="D10" s="344" t="str">
+        <x:v>冷缓存包括序列化/写盘填充成本；热缓存测已填充目录。</x:v>
+      </x:c>
+      <x:c r="E10" s="344"/>
+      <x:c r="F10" s="344"/>
+      <x:c r="G10" s="344"/>
+      <x:c r="H10" s="344"/>
+      <x:c r="I10" s="344"/>
+      <x:c r="J10" s="344"/>
+      <x:c r="K10" s="344"/>
+      <x:c r="L10" s="344"/>
+      <x:c r="M10" s="344"/>
+      <x:c r="N10" s="344"/>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="345" t="str">
+        <x:v>进程 CPU</x:v>
+      </x:c>
+      <x:c r="B11" s="345" t="str">
+        <x:v>-62.1%</x:v>
+      </x:c>
+      <x:c r="C11" s="345" t="str">
+        <x:v>48.6%</x:v>
+      </x:c>
+      <x:c r="D11" s="345" t="str">
+        <x:v>用 process CPU 记录，不是 CPU 配额利用率。</x:v>
+      </x:c>
+      <x:c r="E11" s="345"/>
+      <x:c r="F11" s="345"/>
+      <x:c r="G11" s="345"/>
+      <x:c r="H11" s="345"/>
+      <x:c r="I11" s="345"/>
+      <x:c r="J11" s="345"/>
+      <x:c r="K11" s="345"/>
+      <x:c r="L11" s="345"/>
+      <x:c r="M11" s="345"/>
+      <x:c r="N11" s="345"/>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="345" t="str">
+        <x:v>AST 解析 CPU</x:v>
+      </x:c>
+      <x:c r="B12" s="345" t="str">
+        <x:v>-95.9%</x:v>
+      </x:c>
+      <x:c r="C12" s="345" t="str">
+        <x:v>8.1%</x:v>
+      </x:c>
+      <x:c r="D12" s="345" t="str">
+        <x:v>热缓存解析调用从 9,508 降到 201，命中 9,307。</x:v>
+      </x:c>
+      <x:c r="E12" s="345"/>
+      <x:c r="F12" s="345"/>
+      <x:c r="G12" s="345"/>
+      <x:c r="H12" s="345"/>
+      <x:c r="I12" s="345"/>
+      <x:c r="J12" s="345"/>
+      <x:c r="K12" s="345"/>
+      <x:c r="L12" s="345"/>
+      <x:c r="M12" s="345"/>
+      <x:c r="N12" s="345"/>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="345" t="str">
+        <x:v>Detector 阶段墙钟</x:v>
+      </x:c>
+      <x:c r="B13" s="345" t="str">
+        <x:v>-51.6%</x:v>
+      </x:c>
+      <x:c r="C13" s="345" t="str">
+        <x:v>59.5%</x:v>
+      </x:c>
+      <x:c r="D13" s="345" t="str">
+        <x:v>E2 热跑复用完整结果 13,037 次，另有 107 次 miss 后重算。</x:v>
+      </x:c>
+      <x:c r="E13" s="345"/>
+      <x:c r="F13" s="345"/>
+      <x:c r="G13" s="345"/>
+      <x:c r="H13" s="345"/>
+      <x:c r="I13" s="345"/>
+      <x:c r="J13" s="345"/>
+      <x:c r="K13" s="345"/>
+      <x:c r="L13" s="345"/>
+      <x:c r="M13" s="345"/>
+      <x:c r="N13" s="345"/>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="345" t="str">
+        <x:v>结果复用 source paths</x:v>
+      </x:c>
+      <x:c r="B14" s="345" t="str">
+        <x:v>6,571 paths</x:v>
+      </x:c>
+      <x:c r="C14" s="345" t="str">
+        <x:v>0 paths</x:v>
+      </x:c>
+      <x:c r="D14" s="345" t="str">
+        <x:v>head inventory 的 9,508 个文件仍全部扫描；复用仅作用于声明了安全单文件契约的 detector。</x:v>
+      </x:c>
+      <x:c r="E14" s="345"/>
+      <x:c r="F14" s="345"/>
+      <x:c r="G14" s="345"/>
+      <x:c r="H14" s="345"/>
+      <x:c r="I14" s="345"/>
+      <x:c r="J14" s="345"/>
+      <x:c r="K14" s="345"/>
+      <x:c r="L14" s="345"/>
+      <x:c r="M14" s="345"/>
+      <x:c r="N14" s="345"/>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="345" t="str">
+        <x:v>结果/覆盖</x:v>
+      </x:c>
+      <x:c r="B15" s="345" t="str">
+        <x:v>63 diagnostics; 11/11 等价</x:v>
+      </x:c>
+      <x:c r="C15" s="345" t="str">
+        <x:v>11/11 等价</x:v>
+      </x:c>
+      <x:c r="D15" s="345" t="str">
+        <x:v>E0 与 E2 热缓存签名一致；11 组均 completed_with_limitations，未声称漏洞准确率。</x:v>
+      </x:c>
+      <x:c r="E15" s="345"/>
+      <x:c r="F15" s="345"/>
+      <x:c r="G15" s="345"/>
+      <x:c r="H15" s="345"/>
+      <x:c r="I15" s="345"/>
+      <x:c r="J15" s="345"/>
+      <x:c r="K15" s="345"/>
+      <x:c r="L15" s="345"/>
+      <x:c r="M15" s="345"/>
+      <x:c r="N15" s="345"/>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="346" t="str">
+        <x:v>最大组件 RSS</x:v>
+      </x:c>
+      <x:c r="B16" s="346" t="str">
+        <x:v>61.5%</x:v>
+      </x:c>
+      <x:c r="C16" s="346" t="str">
+        <x:v>62.9%</x:v>
+      </x:c>
+      <x:c r="D16" s="346" t="str">
+        <x:v>按串行组件进程的最大峰值计算；热缓存 RSS 高于 E0，不能宣称内存降低。</x:v>
+      </x:c>
+      <x:c r="E16" s="346"/>
+      <x:c r="F16" s="346"/>
+      <x:c r="G16" s="346"/>
+      <x:c r="H16" s="346"/>
+      <x:c r="I16" s="346"/>
+      <x:c r="J16" s="346"/>
+      <x:c r="K16" s="346"/>
+      <x:c r="L16" s="346"/>
+      <x:c r="M16" s="346"/>
+      <x:c r="N16" s="346"/>
+    </x:row>
+    <x:row r="17" ht="8" customHeight="1">
+      <x:c r="A17" s="347"/>
+      <x:c r="B17" s="347"/>
+      <x:c r="C17" s="347"/>
+      <x:c r="D17" s="347"/>
+      <x:c r="E17" s="347"/>
+      <x:c r="F17" s="347"/>
+      <x:c r="G17" s="347"/>
+      <x:c r="H17" s="347"/>
+      <x:c r="I17" s="347"/>
+      <x:c r="J17" s="347"/>
+      <x:c r="K17" s="347"/>
+      <x:c r="L17" s="347"/>
+      <x:c r="M17" s="347"/>
+      <x:c r="N17" s="347"/>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="348" t="str">
+        <x:v>组件级原始对照：E0 / E2 冷 / E2 热，每行绑定固定 commit、阶段计时、覆盖状态与结果签名。</x:v>
+      </x:c>
+      <x:c r="B18" s="348" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C18" s="348" t="str">
+        <x:v>bbb92dbb2f52aca54ab268307c9476ac1802f3ff</x:v>
+      </x:c>
+      <x:c r="D18" s="349" t="n">
+        <x:v>5.5312</x:v>
+      </x:c>
+      <x:c r="E18" s="349" t="n">
+        <x:v>4.687520999999999</x:v>
+      </x:c>
+      <x:c r="F18" s="349" t="n">
+        <x:v>2.506843992999999</x:v>
+      </x:c>
+      <x:c r="G18" s="349" t="n">
+        <x:v>1.7084219229999462</x:v>
+      </x:c>
+      <x:c r="H18" s="350" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="I18" s="350" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="J18" s="350" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K18" s="348" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L18" s="348" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M18" s="348" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N18" s="348" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="351" t="str">
+        <x:v>组件</x:v>
+      </x:c>
+      <x:c r="B19" s="351" t="str">
+        <x:v>实验组</x:v>
+      </x:c>
+      <x:c r="C19" s="351" t="str">
+        <x:v>固定 head commit</x:v>
+      </x:c>
+      <x:c r="D19" s="352" t="str">
+        <x:v>墙钟秒</x:v>
+      </x:c>
+      <x:c r="E19" s="352" t="str">
+        <x:v>CPU 秒</x:v>
+      </x:c>
+      <x:c r="F19" s="352" t="str">
+        <x:v>AST CPU 秒</x:v>
+      </x:c>
+      <x:c r="G19" s="352" t="str">
+        <x:v>Detector 阶段秒</x:v>
+      </x:c>
+      <x:c r="H19" s="353" t="str">
+        <x:v>扫描文件清单</x:v>
+      </x:c>
+      <x:c r="I19" s="353" t="str">
+        <x:v>Parser 调用</x:v>
+      </x:c>
+      <x:c r="J19" s="353" t="str">
+        <x:v>AST hit</x:v>
+      </x:c>
+      <x:c r="K19" s="351" t="str">
+        <x:v>结果 hit / miss</x:v>
+      </x:c>
+      <x:c r="L19" s="351" t="str">
+        <x:v>候选诊断</x:v>
+      </x:c>
+      <x:c r="M19" s="351" t="str">
+        <x:v>整体 / detector 状态</x:v>
+      </x:c>
+      <x:c r="N19" s="351" t="str">
+        <x:v>与 E0 签名</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="204" t="str">
+        <x:v>communication_ipc</x:v>
+      </x:c>
+      <x:c r="B20" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C20" s="204" t="str">
+        <x:v>bbb92dbb2f52aca54ab268307c9476ac1802f3ff</x:v>
+      </x:c>
+      <x:c r="D20" s="207" t="n">
+        <x:v>5.5312</x:v>
+      </x:c>
+      <x:c r="E20" s="207" t="n">
+        <x:v>4.687520999999999</x:v>
+      </x:c>
+      <x:c r="F20" s="207" t="n">
+        <x:v>2.506843992999999</x:v>
+      </x:c>
+      <x:c r="G20" s="207" t="n">
+        <x:v>1.7084219229999462</x:v>
+      </x:c>
+      <x:c r="H20" s="210" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="I20" s="210" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="J20" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L20" s="204" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M20" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N20" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="204" t="str">
+        <x:v>inputmethod_imf</x:v>
+      </x:c>
+      <x:c r="B21" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C21" s="204" t="str">
+        <x:v>7777cba9eb19085af8e7b90088531028d2937460</x:v>
+      </x:c>
+      <x:c r="D21" s="207" t="n">
+        <x:v>5.7057</x:v>
+      </x:c>
+      <x:c r="E21" s="207" t="n">
+        <x:v>4.937694</x:v>
+      </x:c>
+      <x:c r="F21" s="207" t="n">
+        <x:v>2.046199595000002</x:v>
+      </x:c>
+      <x:c r="G21" s="207" t="n">
+        <x:v>2.462580606000074</x:v>
+      </x:c>
+      <x:c r="H21" s="210" t="n">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="I21" s="210" t="n">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="J21" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K21" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L21" s="204" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M21" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N21" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="204" t="str">
+        <x:v>multimedia_camera_framework</x:v>
+      </x:c>
+      <x:c r="B22" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C22" s="204" t="str">
+        <x:v>085a5d0e2dc1c90a4b676bad55675a1cf12a6380</x:v>
+      </x:c>
+      <x:c r="D22" s="207" t="n">
+        <x:v>18.2618</x:v>
+      </x:c>
+      <x:c r="E22" s="207" t="n">
+        <x:v>17.55388</x:v>
+      </x:c>
+      <x:c r="F22" s="207" t="n">
+        <x:v>5.292039309000004</x:v>
+      </x:c>
+      <x:c r="G22" s="207" t="n">
+        <x:v>11.552708977999941</x:v>
+      </x:c>
+      <x:c r="H22" s="210" t="n">
+        <x:v>1696</x:v>
+      </x:c>
+      <x:c r="I22" s="210" t="n">
+        <x:v>1696</x:v>
+      </x:c>
+      <x:c r="J22" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K22" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L22" s="204" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="M22" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N22" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="204" t="str">
+        <x:v>multimedia_player_framework</x:v>
+      </x:c>
+      <x:c r="B23" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C23" s="204" t="str">
+        <x:v>9f9a285ff489afa66861a85dcc4213336a463b36</x:v>
+      </x:c>
+      <x:c r="D23" s="207" t="n">
+        <x:v>12.3226</x:v>
+      </x:c>
+      <x:c r="E23" s="207" t="n">
+        <x:v>11.622425</x:v>
+      </x:c>
+      <x:c r="F23" s="207" t="n">
+        <x:v>5.744447191999994</x:v>
+      </x:c>
+      <x:c r="G23" s="207" t="n">
+        <x:v>5.117600766999999</x:v>
+      </x:c>
+      <x:c r="H23" s="210" t="n">
+        <x:v>1773</x:v>
+      </x:c>
+      <x:c r="I23" s="210" t="n">
+        <x:v>1773</x:v>
+      </x:c>
+      <x:c r="J23" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K23" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L23" s="204" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="M23" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N23" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="204" t="str">
+        <x:v>notification_common_event_service</x:v>
+      </x:c>
+      <x:c r="B24" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C24" s="204" t="str">
+        <x:v>aaaaf6d10aa8e1f6bd28673f10d5791d7e9c9e3f</x:v>
+      </x:c>
+      <x:c r="D24" s="207" t="n">
+        <x:v>3.6678</x:v>
+      </x:c>
+      <x:c r="E24" s="207" t="n">
+        <x:v>2.78476</x:v>
+      </x:c>
+      <x:c r="F24" s="207" t="n">
+        <x:v>0.8005643759999999</x:v>
+      </x:c>
+      <x:c r="G24" s="207" t="n">
+        <x:v>1.701731979000101</x:v>
+      </x:c>
+      <x:c r="H24" s="210" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="I24" s="210" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="J24" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K24" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L24" s="204" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M24" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N24" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="204" t="str">
+        <x:v>resourceschedule_background_task_mgr</x:v>
+      </x:c>
+      <x:c r="B25" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C25" s="204" t="str">
+        <x:v>cff2ff475e3885ee814651f6a13d7f8a5782efdd</x:v>
+      </x:c>
+      <x:c r="D25" s="207" t="n">
+        <x:v>3.6937</x:v>
+      </x:c>
+      <x:c r="E25" s="207" t="n">
+        <x:v>2.98426</x:v>
+      </x:c>
+      <x:c r="F25" s="207" t="n">
+        <x:v>0.7957635679999996</x:v>
+      </x:c>
+      <x:c r="G25" s="207" t="n">
+        <x:v>1.9004584410000689</x:v>
+      </x:c>
+      <x:c r="H25" s="210" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="I25" s="210" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="J25" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K25" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L25" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M25" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N25" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="204" t="str">
+        <x:v>security_access_token</x:v>
+      </x:c>
+      <x:c r="B26" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C26" s="204" t="str">
+        <x:v>17d88bfb36bea6c9370ba919ac41a22d16dd66b3</x:v>
+      </x:c>
+      <x:c r="D26" s="207" t="n">
+        <x:v>7.4818</x:v>
+      </x:c>
+      <x:c r="E26" s="207" t="n">
+        <x:v>6.694349</x:v>
+      </x:c>
+      <x:c r="F26" s="207" t="n">
+        <x:v>2.4207220440000063</x:v>
+      </x:c>
+      <x:c r="G26" s="207" t="n">
+        <x:v>3.753679712999997</x:v>
+      </x:c>
+      <x:c r="H26" s="210" t="n">
+        <x:v>1249</x:v>
+      </x:c>
+      <x:c r="I26" s="210" t="n">
+        <x:v>1249</x:v>
+      </x:c>
+      <x:c r="J26" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K26" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L26" s="204" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M26" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N26" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="204" t="str">
+        <x:v>telephony_call_manager</x:v>
+      </x:c>
+      <x:c r="B27" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C27" s="204" t="str">
+        <x:v>6638d1b37f278d7ed380d907674820e7467cedf8</x:v>
+      </x:c>
+      <x:c r="D27" s="207" t="n">
+        <x:v>5.5442</x:v>
+      </x:c>
+      <x:c r="E27" s="207" t="n">
+        <x:v>4.846394999999999</x:v>
+      </x:c>
+      <x:c r="F27" s="207" t="n">
+        <x:v>1.4600292430000006</x:v>
+      </x:c>
+      <x:c r="G27" s="207" t="n">
+        <x:v>3.0406865649999872</x:v>
+      </x:c>
+      <x:c r="H27" s="210" t="n">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="I27" s="210" t="n">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="J27" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K27" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L27" s="204" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M27" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N27" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="A28" s="204" t="str">
+        <x:v>update_updateservice</x:v>
+      </x:c>
+      <x:c r="B28" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C28" s="204" t="str">
+        <x:v>e4942a33cc5ed29040e5c720bea3b2a8e4a79221</x:v>
+      </x:c>
+      <x:c r="D28" s="207" t="n">
+        <x:v>1.6624</x:v>
+      </x:c>
+      <x:c r="E28" s="207" t="n">
+        <x:v>0.9870349999999999</x:v>
+      </x:c>
+      <x:c r="F28" s="207" t="n">
+        <x:v>0.20956187199999995</x:v>
+      </x:c>
+      <x:c r="G28" s="207" t="n">
+        <x:v>0.5314844009999433</x:v>
+      </x:c>
+      <x:c r="H28" s="210" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="I28" s="210" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="J28" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K28" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L28" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M28" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N28" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="30" customHeight="1">
+      <x:c r="A29" s="204" t="str">
+        <x:v>window_window_manager</x:v>
+      </x:c>
+      <x:c r="B29" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C29" s="204" t="str">
+        <x:v>8b0d8fe1b973d865904c942c286b3d2a3b9b08e7</x:v>
+      </x:c>
+      <x:c r="D29" s="207" t="n">
+        <x:v>28.4091</x:v>
+      </x:c>
+      <x:c r="E29" s="207" t="n">
+        <x:v>22.769816</x:v>
+      </x:c>
+      <x:c r="F29" s="207" t="n">
+        <x:v>12.12621375999999</x:v>
+      </x:c>
+      <x:c r="G29" s="207" t="n">
+        <x:v>8.023621605000017</x:v>
+      </x:c>
+      <x:c r="H29" s="210" t="n">
+        <x:v>1944</x:v>
+      </x:c>
+      <x:c r="I29" s="210" t="n">
+        <x:v>1944</x:v>
+      </x:c>
+      <x:c r="J29" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K29" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L29" s="204" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M29" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N29" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="30" customHeight="1">
+      <x:c r="A30" s="204" t="str">
+        <x:v>c_utils_pinned_m2</x:v>
+      </x:c>
+      <x:c r="B30" s="204" t="str">
+        <x:v>E0 同环境全量无缓存</x:v>
+      </x:c>
+      <x:c r="C30" s="204" t="str">
+        <x:v>b807d3dadb7dbb7639fe85b3a5f72da18d318da2</x:v>
+      </x:c>
+      <x:c r="D30" s="207" t="n">
+        <x:v>2.5198</x:v>
+      </x:c>
+      <x:c r="E30" s="207" t="n">
+        <x:v>1.768287</x:v>
+      </x:c>
+      <x:c r="F30" s="207" t="n">
+        <x:v>0.48114812199999984</x:v>
+      </x:c>
+      <x:c r="G30" s="207" t="n">
+        <x:v>1.0349641010000141</x:v>
+      </x:c>
+      <x:c r="H30" s="210" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="I30" s="210" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="J30" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K30" s="204" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="L30" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N30" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="A31" s="204" t="str">
+        <x:v>communication_ipc</x:v>
+      </x:c>
+      <x:c r="B31" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C31" s="204" t="str">
+        <x:v>bbb92dbb2f52aca54ab268307c9476ac1802f3ff</x:v>
+      </x:c>
+      <x:c r="D31" s="207" t="n">
+        <x:v>7.6982</x:v>
+      </x:c>
+      <x:c r="E31" s="207" t="n">
+        <x:v>6.1312560000000005</x:v>
+      </x:c>
+      <x:c r="F31" s="207" t="n">
+        <x:v>2.425058357000004</x:v>
+      </x:c>
+      <x:c r="G31" s="207" t="n">
+        <x:v>2.5253038990000007</x:v>
+      </x:c>
+      <x:c r="H31" s="210" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="I31" s="210" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="J31" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K31" s="204" t="str">
+        <x:v>0 / 810</x:v>
+      </x:c>
+      <x:c r="L31" s="204" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M31" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N31" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="30" customHeight="1">
+      <x:c r="A32" s="204" t="str">
+        <x:v>inputmethod_imf</x:v>
+      </x:c>
+      <x:c r="B32" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C32" s="204" t="str">
+        <x:v>7777cba9eb19085af8e7b90088531028d2937460</x:v>
+      </x:c>
+      <x:c r="D32" s="207" t="n">
+        <x:v>7.8319</x:v>
+      </x:c>
+      <x:c r="E32" s="207" t="n">
+        <x:v>6.547984</x:v>
+      </x:c>
+      <x:c r="F32" s="207" t="n">
+        <x:v>1.7936392300000017</x:v>
+      </x:c>
+      <x:c r="G32" s="207" t="n">
+        <x:v>3.2394236829999983</x:v>
+      </x:c>
+      <x:c r="H32" s="210" t="n">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="I32" s="210" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="J32" s="210" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K32" s="204" t="str">
+        <x:v>0 / 1044</x:v>
+      </x:c>
+      <x:c r="L32" s="204" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M32" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N32" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="30" customHeight="1">
+      <x:c r="A33" s="204" t="str">
+        <x:v>multimedia_camera_framework</x:v>
+      </x:c>
+      <x:c r="B33" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C33" s="204" t="str">
+        <x:v>085a5d0e2dc1c90a4b676bad55675a1cf12a6380</x:v>
+      </x:c>
+      <x:c r="D33" s="207" t="n">
+        <x:v>26.0661</x:v>
+      </x:c>
+      <x:c r="E33" s="207" t="n">
+        <x:v>24.133937000000003</x:v>
+      </x:c>
+      <x:c r="F33" s="207" t="n">
+        <x:v>5.411229190000026</x:v>
+      </x:c>
+      <x:c r="G33" s="207" t="n">
+        <x:v>15.226992105999997</x:v>
+      </x:c>
+      <x:c r="H33" s="210" t="n">
+        <x:v>1696</x:v>
+      </x:c>
+      <x:c r="I33" s="210" t="n">
+        <x:v>1695</x:v>
+      </x:c>
+      <x:c r="J33" s="210" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K33" s="204" t="str">
+        <x:v>0 / 2582</x:v>
+      </x:c>
+      <x:c r="L33" s="204" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="M33" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N33" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="30" customHeight="1">
+      <x:c r="A34" s="204" t="str">
+        <x:v>multimedia_player_framework</x:v>
+      </x:c>
+      <x:c r="B34" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C34" s="204" t="str">
+        <x:v>9f9a285ff489afa66861a85dcc4213336a463b36</x:v>
+      </x:c>
+      <x:c r="D34" s="207" t="n">
+        <x:v>17.0097</x:v>
+      </x:c>
+      <x:c r="E34" s="207" t="n">
+        <x:v>15.859328</x:v>
+      </x:c>
+      <x:c r="F34" s="207" t="n">
+        <x:v>5.70873410100002</x:v>
+      </x:c>
+      <x:c r="G34" s="207" t="n">
+        <x:v>6.095604498</x:v>
+      </x:c>
+      <x:c r="H34" s="210" t="n">
+        <x:v>1773</x:v>
+      </x:c>
+      <x:c r="I34" s="210" t="n">
+        <x:v>1749</x:v>
+      </x:c>
+      <x:c r="J34" s="210" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="K34" s="204" t="str">
+        <x:v>0 / 2174</x:v>
+      </x:c>
+      <x:c r="L34" s="204" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="M34" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N34" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="30" customHeight="1">
+      <x:c r="A35" s="204" t="str">
+        <x:v>notification_common_event_service</x:v>
+      </x:c>
+      <x:c r="B35" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C35" s="204" t="str">
+        <x:v>aaaaf6d10aa8e1f6bd28673f10d5791d7e9c9e3f</x:v>
+      </x:c>
+      <x:c r="D35" s="207" t="n">
+        <x:v>5.646</x:v>
+      </x:c>
+      <x:c r="E35" s="207" t="n">
+        <x:v>3.723718</x:v>
+      </x:c>
+      <x:c r="F35" s="207" t="n">
+        <x:v>0.8559137469999978</x:v>
+      </x:c>
+      <x:c r="G35" s="207" t="n">
+        <x:v>2.3111538329999917</x:v>
+      </x:c>
+      <x:c r="H35" s="210" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="I35" s="210" t="n">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="J35" s="210" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K35" s="204" t="str">
+        <x:v>0 / 430</x:v>
+      </x:c>
+      <x:c r="L35" s="204" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M35" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N35" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="204" t="str">
+        <x:v>resourceschedule_background_task_mgr</x:v>
+      </x:c>
+      <x:c r="B36" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C36" s="204" t="str">
+        <x:v>cff2ff475e3885ee814651f6a13d7f8a5782efdd</x:v>
+      </x:c>
+      <x:c r="D36" s="207" t="n">
+        <x:v>4.4242</x:v>
+      </x:c>
+      <x:c r="E36" s="207" t="n">
+        <x:v>3.409837</x:v>
+      </x:c>
+      <x:c r="F36" s="207" t="n">
+        <x:v>0.5948693919999996</x:v>
+      </x:c>
+      <x:c r="G36" s="207" t="n">
+        <x:v>2.4204968000000093</x:v>
+      </x:c>
+      <x:c r="H36" s="210" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="I36" s="210" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="J36" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K36" s="204" t="str">
+        <x:v>0 / 458</x:v>
+      </x:c>
+      <x:c r="L36" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N36" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="30" customHeight="1">
+      <x:c r="A37" s="204" t="str">
+        <x:v>security_access_token</x:v>
+      </x:c>
+      <x:c r="B37" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C37" s="204" t="str">
+        <x:v>17d88bfb36bea6c9370ba919ac41a22d16dd66b3</x:v>
+      </x:c>
+      <x:c r="D37" s="207" t="n">
+        <x:v>13.6538</x:v>
+      </x:c>
+      <x:c r="E37" s="207" t="n">
+        <x:v>11.409518</x:v>
+      </x:c>
+      <x:c r="F37" s="207" t="n">
+        <x:v>2.833946224999986</x:v>
+      </x:c>
+      <x:c r="G37" s="207" t="n">
+        <x:v>6.35857603800001</x:v>
+      </x:c>
+      <x:c r="H37" s="210" t="n">
+        <x:v>1249</x:v>
+      </x:c>
+      <x:c r="I37" s="210" t="n">
+        <x:v>1246</x:v>
+      </x:c>
+      <x:c r="J37" s="210" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K37" s="204" t="str">
+        <x:v>0 / 2074</x:v>
+      </x:c>
+      <x:c r="L37" s="204" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M37" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N37" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="204" t="str">
+        <x:v>telephony_call_manager</x:v>
+      </x:c>
+      <x:c r="B38" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C38" s="204" t="str">
+        <x:v>6638d1b37f278d7ed380d907674820e7467cedf8</x:v>
+      </x:c>
+      <x:c r="D38" s="207" t="n">
+        <x:v>8.1089</x:v>
+      </x:c>
+      <x:c r="E38" s="207" t="n">
+        <x:v>6.787589</x:v>
+      </x:c>
+      <x:c r="F38" s="207" t="n">
+        <x:v>1.5905124169999996</x:v>
+      </x:c>
+      <x:c r="G38" s="207" t="n">
+        <x:v>3.8781796079999964</x:v>
+      </x:c>
+      <x:c r="H38" s="210" t="n">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="I38" s="210" t="n">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="J38" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K38" s="204" t="str">
+        <x:v>0 / 762</x:v>
+      </x:c>
+      <x:c r="L38" s="204" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M38" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N38" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="204" t="str">
+        <x:v>update_updateservice</x:v>
+      </x:c>
+      <x:c r="B39" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C39" s="204" t="str">
+        <x:v>e4942a33cc5ed29040e5c720bea3b2a8e4a79221</x:v>
+      </x:c>
+      <x:c r="D39" s="207" t="n">
+        <x:v>2.4508</x:v>
+      </x:c>
+      <x:c r="E39" s="207" t="n">
+        <x:v>1.415756</x:v>
+      </x:c>
+      <x:c r="F39" s="207" t="n">
+        <x:v>0.21918963999999988</x:v>
+      </x:c>
+      <x:c r="G39" s="207" t="n">
+        <x:v>1.013364294000013</x:v>
+      </x:c>
+      <x:c r="H39" s="210" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="I39" s="210" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="J39" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K39" s="204" t="str">
+        <x:v>0 / 408</x:v>
+      </x:c>
+      <x:c r="L39" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M39" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N39" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="A40" s="204" t="str">
+        <x:v>window_window_manager</x:v>
+      </x:c>
+      <x:c r="B40" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C40" s="204" t="str">
+        <x:v>8b0d8fe1b973d865904c942c286b3d2a3b9b08e7</x:v>
+      </x:c>
+      <x:c r="D40" s="207" t="n">
+        <x:v>65.5276</x:v>
+      </x:c>
+      <x:c r="E40" s="207" t="n">
+        <x:v>39.219421</x:v>
+      </x:c>
+      <x:c r="F40" s="207" t="n">
+        <x:v>14.612007864000002</x:v>
+      </x:c>
+      <x:c r="G40" s="207" t="n">
+        <x:v>20.08267781500001</x:v>
+      </x:c>
+      <x:c r="H40" s="210" t="n">
+        <x:v>1944</x:v>
+      </x:c>
+      <x:c r="I40" s="210" t="n">
+        <x:v>1944</x:v>
+      </x:c>
+      <x:c r="J40" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K40" s="204" t="str">
+        <x:v>0 / 2214</x:v>
+      </x:c>
+      <x:c r="L40" s="204" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M40" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N40" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="204" t="str">
+        <x:v>c_utils_pinned_m2</x:v>
+      </x:c>
+      <x:c r="B41" s="204" t="str">
+        <x:v>E2 冷缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C41" s="204" t="str">
+        <x:v>b807d3dadb7dbb7639fe85b3a5f72da18d318da2</x:v>
+      </x:c>
+      <x:c r="D41" s="207" t="n">
+        <x:v>6.2098</x:v>
+      </x:c>
+      <x:c r="E41" s="207" t="n">
+        <x:v>2.686437</x:v>
+      </x:c>
+      <x:c r="F41" s="207" t="n">
+        <x:v>0.5756604170000004</x:v>
+      </x:c>
+      <x:c r="G41" s="207" t="n">
+        <x:v>1.9667492979999963</x:v>
+      </x:c>
+      <x:c r="H41" s="210" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="I41" s="210" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="J41" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K41" s="204" t="str">
+        <x:v>0 / 188</x:v>
+      </x:c>
+      <x:c r="L41" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M41" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N41" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="204" t="str">
+        <x:v>communication_ipc</x:v>
+      </x:c>
+      <x:c r="B42" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C42" s="204" t="str">
+        <x:v>bbb92dbb2f52aca54ab268307c9476ac1802f3ff</x:v>
+      </x:c>
+      <x:c r="D42" s="207" t="n">
+        <x:v>4.6863</x:v>
+      </x:c>
+      <x:c r="E42" s="207" t="n">
+        <x:v>2.283778</x:v>
+      </x:c>
+      <x:c r="F42" s="207" t="n">
+        <x:v>0.8683187129999996</x:v>
+      </x:c>
+      <x:c r="G42" s="207" t="n">
+        <x:v>0.8290622080000016</x:v>
+      </x:c>
+      <x:c r="H42" s="210" t="n">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="I42" s="210" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="J42" s="210" t="n">
+        <x:v>660</x:v>
+      </x:c>
+      <x:c r="K42" s="204" t="str">
+        <x:v>809 / 1</x:v>
+      </x:c>
+      <x:c r="L42" s="204" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M42" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N42" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="204" t="str">
+        <x:v>inputmethod_imf</x:v>
+      </x:c>
+      <x:c r="B43" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C43" s="204" t="str">
+        <x:v>7777cba9eb19085af8e7b90088531028d2937460</x:v>
+      </x:c>
+      <x:c r="D43" s="207" t="n">
+        <x:v>4.637</x:v>
+      </x:c>
+      <x:c r="E43" s="207" t="n">
+        <x:v>1.982211</x:v>
+      </x:c>
+      <x:c r="F43" s="207" t="n">
+        <x:v>0.09856639400000008</x:v>
+      </x:c>
+      <x:c r="G43" s="207" t="n">
+        <x:v>1.2313404930000011</x:v>
+      </x:c>
+      <x:c r="H43" s="210" t="n">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="I43" s="210" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="J43" s="210" t="n">
+        <x:v>674</x:v>
+      </x:c>
+      <x:c r="K43" s="204" t="str">
+        <x:v>1038 / 6</x:v>
+      </x:c>
+      <x:c r="L43" s="204" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M43" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N43" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="30" customHeight="1">
+      <x:c r="A44" s="204" t="str">
+        <x:v>multimedia_camera_framework</x:v>
+      </x:c>
+      <x:c r="B44" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C44" s="204" t="str">
+        <x:v>085a5d0e2dc1c90a4b676bad55675a1cf12a6380</x:v>
+      </x:c>
+      <x:c r="D44" s="207" t="n">
+        <x:v>9.3054</x:v>
+      </x:c>
+      <x:c r="E44" s="207" t="n">
+        <x:v>5.65139</x:v>
+      </x:c>
+      <x:c r="F44" s="207" t="n">
+        <x:v>0.19567416900000056</x:v>
+      </x:c>
+      <x:c r="G44" s="207" t="n">
+        <x:v>3.626280399999999</x:v>
+      </x:c>
+      <x:c r="H44" s="210" t="n">
+        <x:v>1696</x:v>
+      </x:c>
+      <x:c r="I44" s="210" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="J44" s="210" t="n">
+        <x:v>1611</x:v>
+      </x:c>
+      <x:c r="K44" s="204" t="str">
+        <x:v>2554 / 28</x:v>
+      </x:c>
+      <x:c r="L44" s="204" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="M44" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N44" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="204" t="str">
+        <x:v>multimedia_player_framework</x:v>
+      </x:c>
+      <x:c r="B45" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C45" s="204" t="str">
+        <x:v>9f9a285ff489afa66861a85dcc4213336a463b36</x:v>
+      </x:c>
+      <x:c r="D45" s="207" t="n">
+        <x:v>5.5158</x:v>
+      </x:c>
+      <x:c r="E45" s="207" t="n">
+        <x:v>3.781427</x:v>
+      </x:c>
+      <x:c r="F45" s="207" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G45" s="207" t="n">
+        <x:v>1.3077140309999997</x:v>
+      </x:c>
+      <x:c r="H45" s="210" t="n">
+        <x:v>1773</x:v>
+      </x:c>
+      <x:c r="I45" s="210" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J45" s="210" t="n">
+        <x:v>1773</x:v>
+      </x:c>
+      <x:c r="K45" s="204" t="str">
+        <x:v>2152 / 22</x:v>
+      </x:c>
+      <x:c r="L45" s="204" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="M45" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N45" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="30" customHeight="1">
+      <x:c r="A46" s="204" t="str">
+        <x:v>notification_common_event_service</x:v>
+      </x:c>
+      <x:c r="B46" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C46" s="204" t="str">
+        <x:v>aaaaf6d10aa8e1f6bd28673f10d5791d7e9c9e3f</x:v>
+      </x:c>
+      <x:c r="D46" s="207" t="n">
+        <x:v>2.3536</x:v>
+      </x:c>
+      <x:c r="E46" s="207" t="n">
+        <x:v>0.930204</x:v>
+      </x:c>
+      <x:c r="F46" s="207" t="n">
+        <x:v>0.015162242000000076</x:v>
+      </x:c>
+      <x:c r="G46" s="207" t="n">
+        <x:v>0.7038850359999955</x:v>
+      </x:c>
+      <x:c r="H46" s="210" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="I46" s="210" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J46" s="210" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="K46" s="204" t="str">
+        <x:v>425 / 5</x:v>
+      </x:c>
+      <x:c r="L46" s="204" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M46" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N46" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="204" t="str">
+        <x:v>resourceschedule_background_task_mgr</x:v>
+      </x:c>
+      <x:c r="B47" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C47" s="204" t="str">
+        <x:v>cff2ff475e3885ee814651f6a13d7f8a5782efdd</x:v>
+      </x:c>
+      <x:c r="D47" s="207" t="n">
+        <x:v>3.0874</x:v>
+      </x:c>
+      <x:c r="E47" s="207" t="n">
+        <x:v>1.741012</x:v>
+      </x:c>
+      <x:c r="F47" s="207" t="n">
+        <x:v>0.026607538999999986</x:v>
+      </x:c>
+      <x:c r="G47" s="207" t="n">
+        <x:v>1.532527180999999</x:v>
+      </x:c>
+      <x:c r="H47" s="210" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="I47" s="210" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J47" s="210" t="n">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="K47" s="204" t="str">
+        <x:v>451 / 7</x:v>
+      </x:c>
+      <x:c r="L47" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M47" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N47" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="30" customHeight="1">
+      <x:c r="A48" s="204" t="str">
+        <x:v>security_access_token</x:v>
+      </x:c>
+      <x:c r="B48" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C48" s="204" t="str">
+        <x:v>17d88bfb36bea6c9370ba919ac41a22d16dd66b3</x:v>
+      </x:c>
+      <x:c r="D48" s="207" t="n">
+        <x:v>4.3393</x:v>
+      </x:c>
+      <x:c r="E48" s="207" t="n">
+        <x:v>2.3621079999999997</x:v>
+      </x:c>
+      <x:c r="F48" s="207" t="n">
+        <x:v>0.01805733599999995</x:v>
+      </x:c>
+      <x:c r="G48" s="207" t="n">
+        <x:v>1.209685002999997</x:v>
+      </x:c>
+      <x:c r="H48" s="210" t="n">
+        <x:v>1249</x:v>
+      </x:c>
+      <x:c r="I48" s="210" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J48" s="210" t="n">
+        <x:v>1244</x:v>
+      </x:c>
+      <x:c r="K48" s="204" t="str">
+        <x:v>2067 / 7</x:v>
+      </x:c>
+      <x:c r="L48" s="204" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M48" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N48" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="30" customHeight="1">
+      <x:c r="A49" s="204" t="str">
+        <x:v>telephony_call_manager</x:v>
+      </x:c>
+      <x:c r="B49" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C49" s="204" t="str">
+        <x:v>6638d1b37f278d7ed380d907674820e7467cedf8</x:v>
+      </x:c>
+      <x:c r="D49" s="207" t="n">
+        <x:v>3.3617</x:v>
+      </x:c>
+      <x:c r="E49" s="207" t="n">
+        <x:v>1.5183740000000001</x:v>
+      </x:c>
+      <x:c r="F49" s="207" t="n">
+        <x:v>0.010103284000000018</x:v>
+      </x:c>
+      <x:c r="G49" s="207" t="n">
+        <x:v>0.9395706019999963</x:v>
+      </x:c>
+      <x:c r="H49" s="210" t="n">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="I49" s="210" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J49" s="210" t="n">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="K49" s="204" t="str">
+        <x:v>752 / 10</x:v>
+      </x:c>
+      <x:c r="L49" s="204" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M49" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N49" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="30" customHeight="1">
+      <x:c r="A50" s="204" t="str">
+        <x:v>update_updateservice</x:v>
+      </x:c>
+      <x:c r="B50" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C50" s="204" t="str">
+        <x:v>e4942a33cc5ed29040e5c720bea3b2a8e4a79221</x:v>
+      </x:c>
+      <x:c r="D50" s="207" t="n">
+        <x:v>2.0081</x:v>
+      </x:c>
+      <x:c r="E50" s="207" t="n">
+        <x:v>0.5838</x:v>
+      </x:c>
+      <x:c r="F50" s="207" t="n">
+        <x:v>0.0024551720000000055</x:v>
+      </x:c>
+      <x:c r="G50" s="207" t="n">
+        <x:v>0.5936570619999983</x:v>
+      </x:c>
+      <x:c r="H50" s="210" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="I50" s="210" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J50" s="210" t="n">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="K50" s="204" t="str">
+        <x:v>408 / 0</x:v>
+      </x:c>
+      <x:c r="L50" s="204" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M50" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N50" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="30" customHeight="1">
+      <x:c r="A51" s="204" t="str">
+        <x:v>window_window_manager</x:v>
+      </x:c>
+      <x:c r="B51" s="204" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C51" s="204" t="str">
+        <x:v>8b0d8fe1b973d865904c942c286b3d2a3b9b08e7</x:v>
+      </x:c>
+      <x:c r="D51" s="207" t="n">
+        <x:v>25.3495</x:v>
+      </x:c>
+      <x:c r="E51" s="207" t="n">
+        <x:v>9.518446</x:v>
+      </x:c>
+      <x:c r="F51" s="207" t="n">
+        <x:v>0.1570310889999999</x:v>
+      </x:c>
+      <x:c r="G51" s="207" t="n">
+        <x:v>7.159777035000005</x:v>
+      </x:c>
+      <x:c r="H51" s="210" t="n">
+        <x:v>1944</x:v>
+      </x:c>
+      <x:c r="I51" s="210" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J51" s="210" t="n">
+        <x:v>1917</x:v>
+      </x:c>
+      <x:c r="K51" s="204" t="str">
+        <x:v>2195 / 19</x:v>
+      </x:c>
+      <x:c r="L51" s="204" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M51" s="204" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N51" s="204" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="30" customHeight="1">
+      <x:c r="A52" s="205" t="str">
+        <x:v>c_utils_pinned_m2</x:v>
+      </x:c>
+      <x:c r="B52" s="205" t="str">
+        <x:v>E2 热缓存（ext4）</x:v>
+      </x:c>
+      <x:c r="C52" s="205" t="str">
+        <x:v>b807d3dadb7dbb7639fe85b3a5f72da18d318da2</x:v>
+      </x:c>
+      <x:c r="D52" s="208" t="n">
+        <x:v>1.9738</x:v>
+      </x:c>
+      <x:c r="E52" s="208" t="n">
+        <x:v>0.597</x:v>
+      </x:c>
+      <x:c r="F52" s="208" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G52" s="208" t="n">
+        <x:v>0.6213675089999953</x:v>
+      </x:c>
+      <x:c r="H52" s="211" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="I52" s="211" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J52" s="211" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="K52" s="205" t="str">
+        <x:v>186 / 2</x:v>
+      </x:c>
+      <x:c r="L52" s="205" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M52" s="205" t="str">
+        <x:v>completed_with_limitations / partial</x:v>
+      </x:c>
+      <x:c r="N52" s="205" t="str">
+        <x:v>一致</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
+    <x:mergeCell ref="D10:N10"/>
+    <x:mergeCell ref="D11:N11"/>
+    <x:mergeCell ref="D12:N12"/>
+    <x:mergeCell ref="D13:N13"/>
+    <x:mergeCell ref="D14:N14"/>
+    <x:mergeCell ref="D15:N15"/>
+    <x:mergeCell ref="A18:N18"/>
+    <x:mergeCell ref="D16:N16"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>